<commit_message>
restore bible spreadsheets with revised naming scheme
</commit_message>
<xml_diff>
--- a/annotators/team/cc/en/annotated_discourse/doyle_bask.14.xlsx
+++ b/annotators/team/cc/en/annotated_discourse/doyle_bask.14.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0" windowWidth="7060" windowHeight="6010"/>
+    <workbookView activeTab="0" windowWidth="7650" windowHeight="6010"/>
   </bookViews>
   <sheets>
     <sheet name="en" sheetId="1" r:id="rId1"/>
@@ -177,12 +177,6 @@
     <t>hear</t>
   </si>
   <si>
-    <t>(In this moment)</t>
-  </si>
-  <si>
-    <t>could also be after, but “in this moment” underlines the drama</t>
-  </si>
-  <si>
     <t>turn</t>
   </si>
   <si>
@@ -217,6 +211,9 @@
   </si>
   <si>
     <t>[repetition]</t>
+  </si>
+  <si>
+    <t>suddenly</t>
   </si>
   <si>
     <t>leave</t>
@@ -255,16 +252,19 @@
     <t>look</t>
   </si>
   <si>
+    <t>but</t>
+  </si>
+  <si>
     <t>give</t>
+  </si>
+  <si>
+    <t>spring</t>
   </si>
   <si>
     <t>fire</t>
   </si>
   <si>
     <t>broad</t>
-  </si>
-  <si>
-    <t>but</t>
   </si>
   <si>
     <t>be (be dead)</t>
@@ -17719,14 +17719,12 @@
         <is>
           <r>
             <rPr>
-              <rFont val="2"/>
               <sz val="10"/>
             </rPr>
             <t>this is a </t>
           </r>
           <r>
             <rPr>
-              <rFont val="2"/>
               <b val="true"/>
               <sz val="10"/>
             </rPr>
@@ -17734,7 +17732,6 @@
           </r>
           <r>
             <rPr>
-              <rFont val="2"/>
               <sz val="10"/>
             </rPr>
             <t> reason, not a factual</t>
@@ -17807,8 +17804,10 @@
           <t>file://conllu/en/doyle_bask.14.conllu#s48_0</t>
         </is>
       </c>
-      <c r="G50" s="20" t="s">
-        <v>51</v>
+      <c r="G50" s="20" t="inlineStr">
+        <is>
+          <t>(In this moment)</t>
+        </is>
       </c>
       <c r="H50" s="21">
         <v>47</v>
@@ -17816,8 +17815,10 @@
       <c r="I50" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="J50" s="23" t="s">
-        <v>52</v>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>could also be after, but “in this moment” underlines the drama</t>
+        </is>
       </c>
     </row>
     <row r="51" spans="1:16384" customHeight="1" ht="72">
@@ -17911,7 +17912,7 @@
         <v>15</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
@@ -17924,7 +17925,7 @@
         </is>
       </c>
       <c r="G53" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H53" s="21">
         <v>50</v>
@@ -17946,7 +17947,7 @@
         <v>2</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
@@ -17964,7 +17965,7 @@
         </is>
       </c>
       <c r="G54" s="20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H54" s="21">
         <v>51</v>
@@ -17998,7 +17999,7 @@
         </is>
       </c>
       <c r="G55" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H55" s="21">
         <v>52</v>
@@ -18059,7 +18060,7 @@
         <v>18</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
@@ -18116,7 +18117,7 @@
         </is>
       </c>
       <c r="G58" s="20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H58" s="21">
         <v>55</v>
@@ -18234,7 +18235,7 @@
         </is>
       </c>
       <c r="G61" s="20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H61" s="21">
         <v>57</v>
@@ -18259,7 +18260,7 @@
         <v>15</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E62" s="12" t="inlineStr">
         <is>
@@ -18299,7 +18300,7 @@
         <v>15</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
@@ -18312,7 +18313,7 @@
         </is>
       </c>
       <c r="G63" s="20" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H63" s="21">
         <v>60</v>
@@ -18392,13 +18393,12 @@
         <v>62</v>
       </c>
       <c r="I65" s="22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J65" s="24" t="inlineStr">
         <is>
           <r>
             <rPr>
-              <rFont val="2"/>
               <b val="true"/>
               <sz val="10"/>
             </rPr>
@@ -18406,7 +18406,6 @@
           </r>
           <r>
             <rPr>
-              <rFont val="2"/>
               <sz val="10"/>
             </rPr>
             <t> for a consequence</t>
@@ -18458,14 +18457,12 @@
         <is>
           <r>
             <rPr>
-              <rFont val="2"/>
               <sz val="10"/>
             </rPr>
             <t>specific is triggered by explicit </t>
           </r>
           <r>
             <rPr>
-              <rFont val="2"/>
               <b val="true"/>
               <sz val="10"/>
             </rPr>
@@ -18473,7 +18470,6 @@
           </r>
           <r>
             <rPr>
-              <rFont val="2"/>
               <sz val="10"/>
             </rPr>
             <t>, overriding answer</t>
@@ -18633,7 +18629,7 @@
         </is>
       </c>
       <c r="G70" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H70" s="21">
         <v>61</v>
@@ -18658,7 +18654,7 @@
         <v>25</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E71" s="12" t="inlineStr">
         <is>
@@ -18693,7 +18689,7 @@
         <v>12</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
@@ -18714,14 +18710,14 @@
         <v>48</v>
       </c>
       <c r="H72" s="21">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="I72" s="22" t="s">
         <v>44</v>
       </c>
       <c r="J72" s="23" t="inlineStr">
         <is>
-          <t>this elaborates on the position where they wait, linked here with the utterance that describes where they wait</t>
+          <t>this elaborates on the position where they wait</t>
         </is>
       </c>
     </row>
@@ -18751,7 +18747,7 @@
         </is>
       </c>
       <c r="G73" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H73" s="21">
         <v>35</v>
@@ -18791,7 +18787,7 @@
         </is>
       </c>
       <c r="G74" s="20" t="s">
-        <v>23</v>
+        <v>63</v>
       </c>
       <c r="H74" s="21">
         <v>71</v>
@@ -18816,7 +18812,7 @@
         <v>2</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
@@ -18913,7 +18909,7 @@
         <v>68</v>
       </c>
       <c r="I77" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J77" s="23" t="inlineStr">
         <is>
@@ -19005,7 +19001,7 @@
         <v>9</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>3</v>
@@ -19048,7 +19044,7 @@
         <v>15</v>
       </c>
       <c r="D81" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E81" s="12" t="inlineStr">
         <is>
@@ -19083,10 +19079,10 @@
         <v>17</v>
       </c>
       <c r="C82" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D82" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="D82" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="E82" s="12" t="inlineStr">
         <is>
@@ -19147,7 +19143,7 @@
         <v>80</v>
       </c>
       <c r="I83" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J83" s="23" t="inlineStr">
         <is>
@@ -19253,7 +19249,7 @@
         </is>
       </c>
       <c r="G86" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H86" s="21">
         <v>83</v>
@@ -19354,7 +19350,7 @@
         <v>2</v>
       </c>
       <c r="D89" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E89" s="12" t="inlineStr">
         <is>
@@ -19407,7 +19403,7 @@
         </is>
       </c>
       <c r="G90" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H90" s="21">
         <v>87</v>
@@ -19432,7 +19428,7 @@
         <v>2</v>
       </c>
       <c r="D91" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E91" s="12" t="inlineStr">
         <is>
@@ -19474,7 +19470,7 @@
         <v>2</v>
       </c>
       <c r="D92" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E92" s="12" t="inlineStr">
         <is>
@@ -19529,7 +19525,7 @@
         </is>
       </c>
       <c r="G93" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H93" s="21">
         <v>90</v>
@@ -19569,7 +19565,7 @@
         </is>
       </c>
       <c r="G94" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H94" s="21">
         <v>90</v>
@@ -19591,10 +19587,10 @@
         <v>2</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D95" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E95" s="12" t="inlineStr">
         <is>
@@ -19631,7 +19627,7 @@
         <v>3</v>
       </c>
       <c r="C96" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D96" s="7" t="s">
         <v>3</v>
@@ -19647,7 +19643,7 @@
         </is>
       </c>
       <c r="G96" s="20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H96" s="21">
         <v>93</v>
@@ -19665,7 +19661,7 @@
         <v>5</v>
       </c>
       <c r="C97" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
@@ -19725,7 +19721,7 @@
         </is>
       </c>
       <c r="G98" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H98" s="21">
         <v>95</v>
@@ -19746,7 +19742,7 @@
         <v>2</v>
       </c>
       <c r="D99" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E99" s="12" t="inlineStr">
         <is>
@@ -19797,17 +19793,15 @@
         </is>
       </c>
       <c r="G100" s="20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H100" s="21">
         <v>97</v>
       </c>
       <c r="I100" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="J100" s="23" t="s">
-        <v>49</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="J100" s="23"/>
     </row>
     <row r="101" spans="1:16384" customHeight="1" ht="72">
       <c r="A101" s="7">
@@ -19833,7 +19827,7 @@
         </is>
       </c>
       <c r="G101" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H101" s="21">
         <v>98</v>
@@ -19873,7 +19867,7 @@
         </is>
       </c>
       <c r="G102" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H102" s="21">
         <v>99</v>
@@ -19913,7 +19907,7 @@
         </is>
       </c>
       <c r="G103" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H103" s="21">
         <v>100</v>
@@ -19949,7 +19943,7 @@
         </is>
       </c>
       <c r="G104" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H104" s="21">
         <v>101</v>
@@ -19988,20 +19982,18 @@
           <t>file://conllu/en/doyle_bask.14.conllu#s103_0</t>
         </is>
       </c>
-      <c r="G105" s="20" t="inlineStr">
-        <is>
-          <t>suddenly</t>
-        </is>
+      <c r="G105" s="20" t="s">
+        <v>76</v>
       </c>
       <c r="H105" s="21">
         <v>102</v>
       </c>
       <c r="I105" s="22" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="J105" s="23" t="inlineStr">
         <is>
-          <t>successive event</t>
+          <t>but asserted</t>
         </is>
       </c>
     </row>
@@ -20051,10 +20043,8 @@
       <c r="C107" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D107" s="7" t="inlineStr">
-        <is>
-          <t>spring</t>
-        </is>
+      <c r="D107" s="7" t="s">
+        <v>78</v>
       </c>
       <c r="E107" s="12" t="inlineStr">
         <is>
@@ -20126,7 +20116,7 @@
         <v>2</v>
       </c>
       <c r="D109" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E109" s="12" t="inlineStr">
         <is>
@@ -20145,7 +20135,7 @@
         <v>106</v>
       </c>
       <c r="I109" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J109" s="23" t="inlineStr">
         <is>
@@ -20187,7 +20177,7 @@
         <v>107</v>
       </c>
       <c r="I110" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J110" s="23" t="inlineStr">
         <is>
@@ -20221,7 +20211,7 @@
         </is>
       </c>
       <c r="G111" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H111" s="21">
         <v>105</v>
@@ -20281,10 +20271,10 @@
         <v>6</v>
       </c>
       <c r="C113" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D113" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E113" s="12" t="inlineStr">
         <is>
@@ -20297,7 +20287,7 @@
         </is>
       </c>
       <c r="G113" s="20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H113" s="21">
         <v>110</v>
@@ -20367,7 +20357,7 @@
         </is>
       </c>
       <c r="G115" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H115" s="21">
         <v>112</v>
@@ -20403,13 +20393,13 @@
         </is>
       </c>
       <c r="G116" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H116" s="21">
         <v>113</v>
       </c>
       <c r="I116" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J116" s="23" t="inlineStr">
         <is>
@@ -20467,7 +20457,7 @@
         <v>4</v>
       </c>
       <c r="C118" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D118" s="7" t="s">
         <v>30</v>
@@ -20489,7 +20479,7 @@
         <v>115</v>
       </c>
       <c r="I118" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J118" s="23"/>
     </row>
@@ -20519,13 +20509,13 @@
         </is>
       </c>
       <c r="G119" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H119" s="21">
         <v>116</v>
       </c>
       <c r="I119" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J119" s="23" t="inlineStr">
         <is>
@@ -20541,7 +20531,7 @@
         <v>7</v>
       </c>
       <c r="C120" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
@@ -20559,7 +20549,7 @@
         </is>
       </c>
       <c r="G120" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H120" s="21">
         <v>117</v>
@@ -20595,7 +20585,7 @@
         </is>
       </c>
       <c r="G121" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H121" s="21">
         <v>118</v>
@@ -20633,7 +20623,7 @@
         </is>
       </c>
       <c r="G122" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H122" s="21">
         <v>119</v>
@@ -20655,7 +20645,7 @@
         <v>16</v>
       </c>
       <c r="C123" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
@@ -20709,7 +20699,7 @@
         </is>
       </c>
       <c r="G124" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H124" s="21">
         <v>121</v>
@@ -20855,7 +20845,7 @@
         </is>
       </c>
       <c r="G128" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H128" s="21">
         <v>125</v>
@@ -20891,7 +20881,7 @@
         </is>
       </c>
       <c r="G129" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H129" s="21">
         <v>126</v>
@@ -20927,7 +20917,7 @@
         </is>
       </c>
       <c r="G130" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H130" s="21">
         <v>127</v>
@@ -20963,7 +20953,7 @@
         </is>
       </c>
       <c r="G131" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H131" s="21">
         <v>128</v>
@@ -21033,7 +21023,7 @@
         </is>
       </c>
       <c r="G133" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H133" s="21">
         <v>130</v>
@@ -21105,7 +21095,7 @@
         <v>132</v>
       </c>
       <c r="I135" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J135" s="23"/>
     </row>
@@ -21141,7 +21131,7 @@
         <v>123</v>
       </c>
       <c r="I136" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J136" s="23" t="inlineStr">
         <is>
@@ -21251,7 +21241,7 @@
         </is>
       </c>
       <c r="G139" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H139" s="21">
         <v>136</v>
@@ -21603,7 +21593,7 @@
         <v>145</v>
       </c>
       <c r="I148" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J148" s="23" t="inlineStr">
         <is>
@@ -21654,7 +21644,7 @@
         <v>21</v>
       </c>
       <c r="D150" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E150" s="12" t="inlineStr">
         <is>
@@ -21683,7 +21673,7 @@
         <v>6</v>
       </c>
       <c r="C151" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D151" s="7" t="s">
         <v>91</v>
@@ -21733,7 +21723,7 @@
         </is>
       </c>
       <c r="G152" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H152" s="21">
         <v>144</v>
@@ -21758,7 +21748,7 @@
         <v>2</v>
       </c>
       <c r="D153" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E153" s="12" t="inlineStr">
         <is>
@@ -21915,7 +21905,7 @@
         </is>
       </c>
       <c r="G157" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H157" s="21">
         <v>154</v>
@@ -21949,7 +21939,7 @@
         </is>
       </c>
       <c r="G158" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H158" s="21">
         <v>151</v>
@@ -22025,7 +22015,7 @@
         <v>157</v>
       </c>
       <c r="I160" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J160" s="23" t="inlineStr">
         <is>
@@ -22143,7 +22133,7 @@
         <v>160</v>
       </c>
       <c r="I163" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J163" s="23"/>
     </row>
@@ -22179,7 +22169,7 @@
         <v>161</v>
       </c>
       <c r="I164" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J164" s="23" t="inlineStr">
         <is>
@@ -22249,13 +22239,13 @@
         </is>
       </c>
       <c r="G166" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H166" s="21">
         <v>163</v>
       </c>
       <c r="I166" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J166" s="23"/>
     </row>
@@ -22433,7 +22423,7 @@
         </is>
       </c>
       <c r="G171" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H171" s="21">
         <v>168</v>
@@ -22543,7 +22533,7 @@
         </is>
       </c>
       <c r="G174" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H174" s="21">
         <v>169</v>
@@ -22564,7 +22554,7 @@
         <v>15</v>
       </c>
       <c r="D175" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E175" s="12" t="inlineStr">
         <is>
@@ -22577,7 +22567,7 @@
         </is>
       </c>
       <c r="G175" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H175" s="21">
         <v>172</v>
@@ -22613,7 +22603,7 @@
         </is>
       </c>
       <c r="G176" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H176" s="21">
         <v>173</v>
@@ -22741,7 +22731,7 @@
         <v>176</v>
       </c>
       <c r="I179" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J179" s="23"/>
     </row>
@@ -22870,7 +22860,7 @@
         <v>15</v>
       </c>
       <c r="D183" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E183" s="12" t="inlineStr">
         <is>
@@ -22985,7 +22975,7 @@
         <v>5</v>
       </c>
       <c r="C186" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D186" s="7" t="inlineStr">
         <is>
@@ -23226,7 +23216,7 @@
         <v>2</v>
       </c>
       <c r="D192" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E192" s="12" t="inlineStr">
         <is>
@@ -23239,7 +23229,7 @@
         </is>
       </c>
       <c r="G192" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H192" s="21">
         <v>189</v>
@@ -23339,13 +23329,13 @@
         </is>
       </c>
       <c r="G195" s="20" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H195" s="21">
         <v>192</v>
       </c>
       <c r="I195" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J195" s="23" t="inlineStr">
         <is>
@@ -23411,7 +23401,7 @@
         </is>
       </c>
       <c r="G197" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H197" s="21">
         <v>190</v>
@@ -23580,7 +23570,7 @@
         <v>2</v>
       </c>
       <c r="D202" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E202" s="12" t="inlineStr">
         <is>
@@ -23612,7 +23602,7 @@
         <v>2</v>
       </c>
       <c r="D203" s="7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E203" s="12" t="inlineStr">
         <is>
@@ -23625,7 +23615,7 @@
         </is>
       </c>
       <c r="G203" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H203" s="21">
         <v>200</v>
@@ -23736,7 +23726,7 @@
         </is>
       </c>
       <c r="G206" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H206" s="21">
         <v>203</v>
@@ -23772,13 +23762,13 @@
         </is>
       </c>
       <c r="G207" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H207" s="21">
         <v>204</v>
       </c>
       <c r="I207" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J207" s="23"/>
     </row>
@@ -23865,7 +23855,7 @@
         <v>2</v>
       </c>
       <c r="D210" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E210" s="12" t="inlineStr">
         <is>
@@ -23878,7 +23868,7 @@
         </is>
       </c>
       <c r="G210" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H210" s="21">
         <v>207</v>
@@ -23928,7 +23918,7 @@
         <v>8</v>
       </c>
       <c r="C212" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D212" s="7" t="inlineStr">
         <is>
@@ -24128,7 +24118,7 @@
         </is>
       </c>
       <c r="G217" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H217" s="21">
         <v>212</v>
@@ -24162,7 +24152,7 @@
         </is>
       </c>
       <c r="G218" s="20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H218" s="21">
         <v>215</v>
@@ -24183,7 +24173,7 @@
         <v>2</v>
       </c>
       <c r="D219" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E219" s="12" t="inlineStr">
         <is>
@@ -24196,7 +24186,7 @@
         </is>
       </c>
       <c r="G219" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H219" s="21">
         <v>216</v>
@@ -24232,7 +24222,7 @@
         </is>
       </c>
       <c r="G220" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H220" s="21">
         <v>217</v>
@@ -24380,7 +24370,7 @@
         </is>
       </c>
       <c r="G224" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H224" s="21">
         <v>219</v>
@@ -24420,7 +24410,7 @@
         <v>222</v>
       </c>
       <c r="I225" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J225" s="23"/>
     </row>
@@ -24468,7 +24458,7 @@
         <v>8</v>
       </c>
       <c r="C227" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D227" s="7" t="inlineStr">
         <is>
@@ -24524,13 +24514,13 @@
         </is>
       </c>
       <c r="G228" s="20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H228" s="21">
         <v>225</v>
       </c>
       <c r="I228" s="22" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="J228" s="23"/>
     </row>
@@ -24585,7 +24575,7 @@
         </is>
       </c>
       <c r="D230" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E230" s="12" t="inlineStr">
         <is>
@@ -24658,7 +24648,7 @@
         <v>10</v>
       </c>
       <c r="C232" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D232" s="7" t="inlineStr">
         <is>
@@ -24850,7 +24840,7 @@
         <v>2</v>
       </c>
       <c r="D237" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E237" s="12" t="inlineStr">
         <is>
@@ -24863,7 +24853,7 @@
         </is>
       </c>
       <c r="G237" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H237" s="21">
         <v>233</v>
@@ -24899,7 +24889,7 @@
         </is>
       </c>
       <c r="G238" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H238" s="21">
         <v>223</v>
@@ -24942,7 +24932,7 @@
         </is>
       </c>
       <c r="G239" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H239" s="21">
         <v>235</v>
@@ -24982,7 +24972,7 @@
         </is>
       </c>
       <c r="G240" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H240" s="21">
         <v>237</v>
@@ -25028,7 +25018,7 @@
         <v>238</v>
       </c>
       <c r="I241" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J241" s="23"/>
     </row>
@@ -25092,7 +25082,7 @@
         </is>
       </c>
       <c r="G243" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H243" s="21">
         <v>239</v>
@@ -25113,7 +25103,7 @@
         <v>2</v>
       </c>
       <c r="D244" s="7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E244" s="12" t="inlineStr">
         <is>
@@ -25126,7 +25116,7 @@
         </is>
       </c>
       <c r="G244" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H244" s="21">
         <v>241</v>
@@ -25496,7 +25486,7 @@
         </is>
       </c>
       <c r="G254" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H254" s="21">
         <v>251</v>
@@ -25570,7 +25560,7 @@
         </is>
       </c>
       <c r="G256" s="20" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="H256" s="21">
         <v>252</v>
@@ -25592,7 +25582,7 @@
         <v>12</v>
       </c>
       <c r="C257" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D257" s="7" t="inlineStr">
         <is>
@@ -25698,7 +25688,7 @@
         <v>254</v>
       </c>
       <c r="I259" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J259" s="23" t="inlineStr">
         <is>
@@ -25738,7 +25728,7 @@
         <v>257</v>
       </c>
       <c r="I260" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J260" s="23"/>
     </row>
@@ -25814,7 +25804,7 @@
         <v>259</v>
       </c>
       <c r="I262" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J262" s="23"/>
     </row>
@@ -26002,7 +25992,7 @@
         <v>264</v>
       </c>
       <c r="I267" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J267" s="23" t="inlineStr">
         <is>
@@ -26042,7 +26032,7 @@
         <v>265</v>
       </c>
       <c r="I268" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J268" s="23" t="inlineStr">
         <is>
@@ -26286,7 +26276,7 @@
         <v>271</v>
       </c>
       <c r="I274" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J274" s="23" t="inlineStr">
         <is>

</xml_diff>